<commit_message>
Speed up employee list filters and add Campus/Dept/Category filters.
Avoid blocking live-table refreshes with deferred ISKOLARIS sync and early session lock release; trim list queries and permissions for faster AJAX reloads.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/templates/employee_salary_upload_template.xlsx
+++ b/resources/templates/employee_salary_upload_template.xlsx
@@ -472,7 +472,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:P150"/>
+  <dimension ref="A1:P154"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:16">
@@ -3247,6 +3247,78 @@
       <c r="O150" s="1"/>
       <c r="P150" s="1"/>
     </row>
+    <row r="151" spans="1:16">
+      <c r="A151" s="1"/>
+      <c r="B151" s="1"/>
+      <c r="C151" s="1"/>
+      <c r="D151" s="1"/>
+      <c r="E151" s="1"/>
+      <c r="F151" s="1"/>
+      <c r="G151" s="1"/>
+      <c r="H151" s="1"/>
+      <c r="I151" s="1"/>
+      <c r="J151" s="1"/>
+      <c r="K151" s="1"/>
+      <c r="L151" s="1"/>
+      <c r="M151" s="1"/>
+      <c r="N151" s="1"/>
+      <c r="O151" s="1"/>
+      <c r="P151" s="1"/>
+    </row>
+    <row r="152" spans="1:16">
+      <c r="A152" s="1"/>
+      <c r="B152" s="1"/>
+      <c r="C152" s="1"/>
+      <c r="D152" s="1"/>
+      <c r="E152" s="1"/>
+      <c r="F152" s="1"/>
+      <c r="G152" s="1"/>
+      <c r="H152" s="1"/>
+      <c r="I152" s="1"/>
+      <c r="J152" s="1"/>
+      <c r="K152" s="1"/>
+      <c r="L152" s="1"/>
+      <c r="M152" s="1"/>
+      <c r="N152" s="1"/>
+      <c r="O152" s="1"/>
+      <c r="P152" s="1"/>
+    </row>
+    <row r="153" spans="1:16">
+      <c r="A153" s="1"/>
+      <c r="B153" s="1"/>
+      <c r="C153" s="1"/>
+      <c r="D153" s="1"/>
+      <c r="E153" s="1"/>
+      <c r="F153" s="1"/>
+      <c r="G153" s="1"/>
+      <c r="H153" s="1"/>
+      <c r="I153" s="1"/>
+      <c r="J153" s="1"/>
+      <c r="K153" s="1"/>
+      <c r="L153" s="1"/>
+      <c r="M153" s="1"/>
+      <c r="N153" s="1"/>
+      <c r="O153" s="1"/>
+      <c r="P153" s="1"/>
+    </row>
+    <row r="154" spans="1:16">
+      <c r="A154" s="1"/>
+      <c r="B154" s="1"/>
+      <c r="C154" s="1"/>
+      <c r="D154" s="1"/>
+      <c r="E154" s="1"/>
+      <c r="F154" s="1"/>
+      <c r="G154" s="1"/>
+      <c r="H154" s="1"/>
+      <c r="I154" s="1"/>
+      <c r="J154" s="1"/>
+      <c r="K154" s="1"/>
+      <c r="L154" s="1"/>
+      <c r="M154" s="1"/>
+      <c r="N154" s="1"/>
+      <c r="O154" s="1"/>
+      <c r="P154" s="1"/>
+    </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>